<commit_message>
fix:auto detect and capture
</commit_message>
<xml_diff>
--- a/backend/exports/2026-05-13/visitors.xlsx
+++ b/backend/exports/2026-05-13/visitors.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="39">
   <si>
     <t>id</t>
   </si>
@@ -82,91 +82,52 @@
     <t>Abdul Rehman</t>
   </si>
   <si>
+    <t>15013-2553761-1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>THE MAGNUM ICE CREAM COMPANY</t>
+  </si>
+  <si>
+    <t>2026-05-13T07:29:46.000Z</t>
+  </si>
+  <si>
+    <t>/uploads/visitors/2026-05-13/1778657357200-73695674.jpg</t>
+  </si>
+  <si>
+    <t>/uploads/cnic-front/2026-05-13/1778657365686-435836760.jpg</t>
+  </si>
+  <si>
+    <t>GP-20260513-0002</t>
+  </si>
+  <si>
+    <t>RA . Abdul Rehman</t>
+  </si>
+  <si>
     <t>34501-3255376-1</t>
   </si>
   <si>
-    <t>M Nawaz</t>
-  </si>
-  <si>
-    <t>03456666052</t>
-  </si>
-  <si>
-    <t>AivraSol</t>
-  </si>
-  <si>
-    <t>awais</t>
-  </si>
-  <si>
-    <t>CS</t>
-  </si>
-  <si>
-    <t>Meeting</t>
-  </si>
-  <si>
-    <t>5730</t>
-  </si>
-  <si>
-    <t>Main Gate</t>
-  </si>
-  <si>
-    <t>2026-05-12T20:43:33.000Z</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>/uploads/cnic-front/2026-05-13/1778618392591-176713425.jpg</t>
-  </si>
-  <si>
-    <t>/uploads/cnic-back/2026-05-13/1778618229092-679525047.jpg</t>
-  </si>
-  <si>
-    <t>GP-20260513-0002</t>
-  </si>
-  <si>
-    <t>DIGI Logs</t>
-  </si>
-  <si>
-    <t>2026-05-12T21:04:19.000Z</t>
-  </si>
-  <si>
-    <t>/uploads/visitors/2026-05-13/1778619850800-73927545.jpg</t>
-  </si>
-  <si>
-    <t>/uploads/cnic-front/2026-05-13/1778619800390-648644793.jpg</t>
-  </si>
-  <si>
-    <t>/uploads/cnic-back/2026-05-13/1778619238943-845457225.jpg</t>
+    <t>2026-05-13T08:40:41.000Z</t>
+  </si>
+  <si>
+    <t>/uploads/visitors/2026-05-13/1778661618906-154908780.jpg</t>
+  </si>
+  <si>
+    <t>/uploads/cnic-front/2026-05-13/1778661629052-351539172.jpg</t>
   </si>
   <si>
     <t>GP-20260513-0003</t>
   </si>
   <si>
-    <t>Muhammad Awais -</t>
-  </si>
-  <si>
-    <t>34503-0396530-3</t>
-  </si>
-  <si>
-    <t>AivraSol Digital Solutions</t>
-  </si>
-  <si>
-    <t>2026-05-12T21:11:11.000Z</t>
-  </si>
-  <si>
-    <t>/uploads/visitors/2026-05-13/1778620264437-190979278.jpg</t>
-  </si>
-  <si>
-    <t>/uploads/cnic-front/2026-05-13/1778620205646-799470526.jpg</t>
-  </si>
-  <si>
-    <t>GP-20260513-0004</t>
-  </si>
-  <si>
-    <t>2026-05-12T21:17:28.000Z</t>
-  </si>
-  <si>
-    <t>/uploads/cnic-front/2026-05-13/1778620602638-540521783.jpg</t>
+    <t>2026-05-13T08:48:08.000Z</t>
+  </si>
+  <si>
+    <t>/uploads/visitors/2026-05-13/1778662023837-568101333.jpg</t>
+  </si>
+  <si>
+    <t>/uploads/cnic-front/2026-05-13/1778662032058-130460436.jpg</t>
   </si>
 </sst>
 </file>
@@ -543,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="21" width="18" customWidth="1"/>
@@ -631,52 +592,52 @@
         <v>24</v>
       </c>
       <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" t="s">
         <v>26</v>
       </c>
-      <c r="H2" t="s">
+      <c r="N2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" t="s">
+      <c r="Q2" t="s">
         <v>28</v>
       </c>
-      <c r="J2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>34</v>
-      </c>
       <c r="R2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="T2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
@@ -684,64 +645,64 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" t="s">
+        <v>24</v>
+      </c>
+      <c r="P3" t="s">
         <v>33</v>
       </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" t="s">
-        <v>38</v>
-      </c>
-      <c r="N3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P3" t="s">
-        <v>39</v>
-      </c>
       <c r="Q3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R3" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="T3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="U3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
@@ -749,129 +710,64 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="K4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="L4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="M4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="N4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="P4" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="Q4" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="R4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="T4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="U4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" t="s">
-        <v>33</v>
-      </c>
-      <c r="P5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>51</v>
-      </c>
-      <c r="R5" t="s">
-        <v>33</v>
-      </c>
-      <c r="S5" t="s">
-        <v>33</v>
-      </c>
-      <c r="T5" t="s">
-        <v>50</v>
-      </c>
-      <c r="U5" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>